<commit_message>
Reports auto update (member)
</commit_message>
<xml_diff>
--- a/reports/member_funnel/downloads/member_funnel_1d_non_buyer.xlsx
+++ b/reports/member_funnel/downloads/member_funnel_1d_non_buyer.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>greatx0001</t>
+          <t>cgkrry</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01054162411</t>
+          <t>01085513271</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>98307</t>
+          <t>48578</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>EDM_0329</t>
+          <t>KAKAO_alimtalk</t>
         </is>
       </c>
     </row>
@@ -500,233 +500,233 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>lefy</t>
+          <t>kk_4222073058</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>01022414020</t>
+          <t>01046077586</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>23592</t>
+          <t>272870</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>[PF]A+SC_상시(1865MF,구매+장바구니)</t>
+          <t>KAKAO_CH_event</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ju7464</t>
+          <t>kk_2873136069</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>01035397467</t>
+          <t>01048866068</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>18502</t>
+          <t>213981</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[PF]전환_상시(2565MF,비구매자14일)</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>kk_3835565251</t>
+          <t>iloveyoutoo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01027409786</t>
+          <t>01050563632</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>263950</t>
+          <t>52960</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>goodphm69</t>
+          <t>kk_3471972251</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>01096632959</t>
+          <t>01091336229</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>305966</t>
+          <t>244043</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Organic Traffic</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Organic Traffic</t>
+          <t>naver_brandsearch_mobile</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>lego81</t>
+          <t>kk_4891271476</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>01028604947</t>
+          <t>01042650212</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>139122</t>
+          <t>305956</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Official SNS</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>KAKAO_alimtalk</t>
+          <t>(referral)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>kk_4931515112</t>
+          <t>kk_4621012084</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>01091232643</t>
+          <t>01029131062</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>307244</t>
+          <t>290948</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>bizboard</t>
+          <t>LMS_ECOM_0501</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>kk_3233598346</t>
+          <t>kingjo</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>01034665375</t>
+          <t>01062660099</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>233814</t>
+          <t>305676</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>KAKAO_CH_MESSAGE_0521_BAHAMA1</t>
+          <t>sa</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>swd71</t>
+          <t>kk_3233598346</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>01071953545</t>
+          <t>01034665375</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>122866</t>
+          <t>233814</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>naver_brandsearch_mobile</t>
+          <t>KAKAO_CH_MESSAGE_0521_BAHAMA1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>wooa8707</t>
+          <t>bcc12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>01091608707</t>
+          <t>01038010281</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>134632</t>
+          <t>132808</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -736,24 +736,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>[PF]A SC_상시(1865MF,논타겟)</t>
+          <t>Paid Ad</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>kk_4933331505</t>
+          <t>nahyun130</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>01038927131</t>
+          <t>01095601814</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>307306</t>
+          <t>303217</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -763,78 +763,78 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>(organic)</t>
+          <t>naver_brandsearch_mobile</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>kk_3333111023</t>
+          <t>kk_4929345311</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>01046548483</t>
+          <t>01047465513</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>238778</t>
+          <t>307178</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0214_newyear</t>
+          <t>[PF_SA] 컬럼비아 상시</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>kk_3357691082</t>
+          <t>jbjjang2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>01038571404</t>
+          <t>01047332579</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>239661</t>
+          <t>140403</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>kk_3008304554</t>
+          <t>swd71</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>01085549546</t>
+          <t>01071953545</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>218985</t>
+          <t>122866</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -844,24 +844,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>[PF]전환_회원가입(유사)</t>
+          <t>naver_brandsearch_mobile</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>yoichi</t>
+          <t>prinseo83</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>01072692907</t>
+          <t>01094532501</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>197150</t>
+          <t>307370</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -878,98 +878,98 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>kk_3886826642</t>
+          <t>kk_4930577896</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>01025882826</t>
+          <t>01026735477</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>267196</t>
+          <t>307224</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>[PF]전환_상시(2565MF,비구매자30일)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>kk_4515845815</t>
+          <t>kjw6636</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>01057985790</t>
+          <t>01091317783</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>285962</t>
+          <t>230429</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>demendgen</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>s5745622</t>
+          <t>mjsf712</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>01056694232</t>
+          <t>01029810334</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>117815</t>
+          <t>105418</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0501</t>
+          <t>0520</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>yagh19</t>
+          <t>kk_3949933982</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>01029169042</t>
+          <t>01026968241</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>55954</t>
+          <t>269859</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -979,51 +979,51 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>KAKAO_CH_MESSAGE_0423_WINDBREAKER</t>
+          <t>KAKAO_CH_event</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>kk_2819656487</t>
+          <t>kk_4925725941</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>01031612454</t>
+          <t>01032250101</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>212399</t>
+          <t>307025</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>120250039724090385</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>kk_4848752733</t>
+          <t>chsyli</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>01090534422</t>
+          <t>01087008003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>304540</t>
+          <t>307275</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1033,51 +1033,51 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>naver_brandsearch_mobile</t>
+          <t>da</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>kk_4925033358</t>
+          <t>haesongey</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>01029288597</t>
+          <t>01062439541</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>306992</t>
+          <t>162716</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>미분류</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>kk_4917287780</t>
+          <t>kk_3866141775</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>01048475995</t>
+          <t>01038425687</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>306708</t>
+          <t>265983</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1087,186 +1087,186 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>[PF]전환_상시(2565MF,비구매자14일)</t>
+          <t>naversa_mo</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>kk_4923488740</t>
+          <t>kk_3464483825</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>01063427194</t>
+          <t>01038526065</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>306937</t>
+          <t>243670</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Official SNS</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>etc</t>
+          <t>(referral)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>aceykh</t>
+          <t>kk_3856109018</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>01041402352</t>
+          <t>01050880234</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>140002</t>
+          <t>265397</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>EDM_TOP</t>
+          <t>[PF]전환_상시(2565MF,비구매자30일)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>edelweissy</t>
+          <t>duhi82</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>01036763198</t>
+          <t>01052468809</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>242345</t>
+          <t>161236</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Organic Traffic</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0501</t>
+          <t>LMS_ECOM_0214_newyear</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>kk_3730296016</t>
+          <t>huny</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>01093160806</t>
+          <t>01064304258</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>252898</t>
+          <t>306823</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>kk_2810289654</t>
+          <t>kk_4791151667</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>01087743302</t>
+          <t>01062417165</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>211764</t>
+          <t>302066</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>[PF]전환_상시(2565MF,비구매자)</t>
+          <t>미분류</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>s6254511</t>
+          <t>kk_4897891838</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>01082007965</t>
+          <t>01049379119</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>32967</t>
+          <t>306116</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Organic Traffic</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>(organic)</t>
+          <t>[PF]전환_회원가입(유사)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>caia99</t>
+          <t>kk_3661001642</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>01075190829</t>
+          <t>01048742308</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>198463</t>
+          <t>249645</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1276,132 +1276,132 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0520</t>
+          <t>KAKAO_alimtalk</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>kk_4933513607</t>
+          <t>hwt0331</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>01065376070</t>
+          <t>01068921188</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>307315</t>
+          <t>105565</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>[PF_SA] 컬럼비아 상시</t>
+          <t>Owned Channel</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>kk_3890453292</t>
+          <t>kk_2932101359</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>01028088681</t>
+          <t>01044886893</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>267360</t>
+          <t>216107</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>kk_3856109018</t>
+          <t>kk_4910660467</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>01050880234</t>
+          <t>01038202323</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>265397</t>
+          <t>306492</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>[PF]전환_상시(2565MF,비구매자30일)</t>
+          <t>[PF]전환_회원가입(유사)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>kk_2914640570</t>
+          <t>ssunnycat</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>01099720247</t>
+          <t>01071921205</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215650</t>
+          <t>175749</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>0520</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>cyh621</t>
+          <t>lkhagva</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>01081816555</t>
+          <t>01026624998</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>98925</t>
+          <t>24183</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1418,17 +1418,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>wkchoo</t>
+          <t>kk_3864038304</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01022806944</t>
+          <t>01074991784</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>98178</t>
+          <t>265831</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1438,24 +1438,24 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>[PF]전환_카탈로그(1865,관심사_01)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>kk_3587862892</t>
+          <t>kk_4638485597</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>01031993677</t>
+          <t>01085071665</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>246481</t>
+          <t>292263</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1465,51 +1465,51 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>KAKAO_CH_MENU_0423_EFW_COOL_1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>kk_3809188341</t>
+          <t>kk_4911889277</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>01054781901</t>
+          <t>01065063406</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>260837</t>
+          <t>306518</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Owned Channel</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>kk_3859769752</t>
+          <t>kk_3890141512</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>01022048066</t>
+          <t>01091355884</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>265580</t>
+          <t>267350</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1519,78 +1519,78 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>etc</t>
+          <t>KAKAO_alimtalk</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>kk_4926021820</t>
+          <t>kk_4925289975</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>01022896126</t>
+          <t>01086230732</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>307045</t>
+          <t>307008</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>naver_brandsearch_pc</t>
+          <t>pfg</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>bjh4895</t>
+          <t>kk_4929674815</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>01042374895</t>
+          <t>01075264562</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>262903</t>
+          <t>307194</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Organic Traffic</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0214_newyear</t>
+          <t>[PF]전환_회원가입(유사)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>kk_4931528603</t>
+          <t>kk_3487761036</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>01097667895</t>
+          <t>01042294295</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>307246</t>
+          <t>244856</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1600,132 +1600,132 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>[PF]전환_회원가입(유사)</t>
+          <t>LMS_ECOM_familycoupon</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>seungrok2</t>
+          <t>rokmc1809</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>01075577530</t>
+          <t>01048841740</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>189140</t>
+          <t>157342</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>KAKAO_CH_event</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>kk_3762729519</t>
+          <t>kk_4619571493</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>01049313705</t>
+          <t>01068999326</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>254890</t>
+          <t>290856</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Owned Channel</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>harlay66</t>
+          <t>kk_3604950061</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>01046663772</t>
+          <t>01090990572</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>163760</t>
+          <t>247196</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>LMS_ECOM</t>
+          <t>da</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>mino606</t>
+          <t>kk_4932866673</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>01032397154</t>
+          <t>01080258100</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>285817</t>
+          <t>307292</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0214_newyear</t>
+          <t>naversa_mo</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>kk_3604950061</t>
+          <t>kk_3809188341</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>01090990572</t>
+          <t>01054781901</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>247196</t>
+          <t>260837</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1735,24 +1735,24 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>naver_brandsearch_mobile</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>kk_4912807536</t>
+          <t>kk_3821813414</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>01046055617</t>
+          <t>01097158512</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>306543</t>
+          <t>262808</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1762,51 +1762,51 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>gdn</t>
+          <t>KAKAO_CH_MENU_0226_TRAILRUN</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>j31goyung</t>
+          <t>kk_4294789203</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>01049366682</t>
+          <t>01071882418</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>16017</t>
+          <t>276147</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0214_newyear</t>
+          <t>미분류</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>kk_4286220576</t>
+          <t>kk_4933800415</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>01053587782</t>
+          <t>01091874163</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>275624</t>
+          <t>307330</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1816,24 +1816,24 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>LMS_ECOM_200416_seasonoff</t>
+          <t>bizboard</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>mc7rap</t>
+          <t>kk_4935843618</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>01085277847</t>
+          <t>01094581578</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>62431</t>
+          <t>307396</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1850,314 +1850,314 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>chyh179</t>
+          <t>legion04</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>01046438047</t>
+          <t>01023174919</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>173234</t>
+          <t>285212</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>KAKAO_CH_MESSAGE_0226_TITANIUM</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>haesongey</t>
+          <t>bbrucelee</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>01062439541</t>
+          <t>01042041669</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>162716</t>
+          <t>165531</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>etc</t>
+          <t>da</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ejilee</t>
+          <t>kk_4935787617</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>01099787850</t>
+          <t>01038091869</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>227362</t>
+          <t>307395</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>etc</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>hiroyys</t>
+          <t>jsy90</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>01042269861</t>
+          <t>01055153689</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>281511</t>
+          <t>304378</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>LMS_ECOM_0410pants2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>kk_4933978970</t>
+          <t>forenet7510</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>01034127366</t>
+          <t>01075071709</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>307342</t>
+          <t>182466</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>미분류</t>
+          <t>KAKAO_CH_MESSAGE_0226_GOODBYEWINTER</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>kk_2879154825</t>
+          <t>kk_4935744011</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>01023371226</t>
+          <t>01038406556</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>214442</t>
+          <t>307392</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>etc</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>imok2000</t>
+          <t>kk_4931694836</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>01087713706</t>
+          <t>01038652226</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>138981</t>
+          <t>307252</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>0520</t>
+          <t>naversa_mo</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>yandk1013</t>
+          <t>k403chy</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>01030048032</t>
+          <t>01037883713</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>111080</t>
+          <t>248753</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>kk_4930023646</t>
+          <t>kim064921</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>01031343144</t>
+          <t>01082310324</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>307208</t>
+          <t>250276</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>(referral)</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>kk_4301842647</t>
+          <t>telecom43</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>01040553470</t>
+          <t>01050853339</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>276610</t>
+          <t>45224</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0214_newyear</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>sky622</t>
+          <t>lentus</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>01066740126</t>
+          <t>01047845080</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>172311</t>
+          <t>217552</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Email_mkt</t>
+          <t>LMS_ECOM_0214_newyear</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>kk_4619229910</t>
+          <t>enddl7072</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>01085180597</t>
+          <t>01067507072</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>290825</t>
+          <t>239652</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2174,108 +2174,324 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>kk_3184496842</t>
+          <t>kk_4933858898</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>01073970916</t>
+          <t>01055972052</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>229003</t>
+          <t>307334</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>(referral)</t>
+          <t>naver_brandsearch_mobile</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>kk_3959996271</t>
+          <t>kk_4285120144</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>01052317543</t>
+          <t>01047588664</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>270350</t>
+          <t>275561</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>(organic)</t>
+          <t>Direct</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>milk1182018</t>
+          <t>kk_4881400849</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>01038657820</t>
+          <t>01057570506</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>289522</t>
+          <t>305635</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>(organic)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>tsc00064</t>
+          <t>kk_4703862679</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>01046567223</t>
+          <t>01099693770</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>141377</t>
+          <t>296141</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>etc</t>
+          <t>Paid Ad</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>panjaok</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>01027564033</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>305598</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Owned Channel</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>(referral)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>kk_3181239874</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>01066774807</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>226780</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>kk_3734762283</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>01071343306</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>253238</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>kk_4705038378</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>01093741585</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>296192</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Paid Ad</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Paid Ad</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>kk_4346815515</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>01087150350</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>279125</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Owned Channel</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>KAKAO_alimtalk</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>yournagel88</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>01094611064</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>182579</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Owned Channel</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Owned Channel</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>efsonata2002</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>01047330993</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>289626</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Owned Channel</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LMS_ECOM_0214_newyear</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>kk_4483674708</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>01067898761</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>284422</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Direct</t>
         </is>
       </c>
     </row>

</xml_diff>